<commit_message>
replace flooding data from matt
</commit_message>
<xml_diff>
--- a/data-raw/CLIMATE_BG20.xlsx
+++ b/data-raw/CLIMATE_BG20.xlsx
@@ -9458,8 +9458,12 @@
       <c r="C37" t="n">
         <v>0.06</v>
       </c>
-      <c r="D37"/>
-      <c r="E37"/>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
       <c r="F37" t="n">
         <v>8.21</v>
       </c>
@@ -9568,8 +9572,12 @@
       <c r="C40" t="n">
         <v>0.094</v>
       </c>
-      <c r="D40"/>
-      <c r="E40"/>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
       <c r="F40" t="n">
         <v>6.69</v>
       </c>
@@ -9754,8 +9762,12 @@
       <c r="C45" t="n">
         <v>0.089</v>
       </c>
-      <c r="D45"/>
-      <c r="E45"/>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
       <c r="F45" t="n">
         <v>15.95</v>
       </c>
@@ -9788,8 +9800,12 @@
       <c r="C46" t="n">
         <v>0.086</v>
       </c>
-      <c r="D46"/>
-      <c r="E46"/>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
       <c r="F46" t="n">
         <v>6.19</v>
       </c>
@@ -10012,8 +10028,12 @@
       <c r="C52" t="n">
         <v>0.118</v>
       </c>
-      <c r="D52"/>
-      <c r="E52"/>
+      <c r="D52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
       <c r="F52" t="n">
         <v>7.32</v>
       </c>
@@ -10122,8 +10142,12 @@
       <c r="C55" t="n">
         <v>0.116</v>
       </c>
-      <c r="D55"/>
-      <c r="E55"/>
+      <c r="D55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
       <c r="F55" t="n">
         <v>7.85</v>
       </c>
@@ -10156,8 +10180,12 @@
       <c r="C56" t="n">
         <v>0.067</v>
       </c>
-      <c r="D56"/>
-      <c r="E56"/>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
+      </c>
       <c r="F56" t="n">
         <v>8.05</v>
       </c>
@@ -10304,8 +10332,12 @@
       <c r="C60" t="n">
         <v>0.11</v>
       </c>
-      <c r="D60"/>
-      <c r="E60"/>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
       <c r="F60" t="n">
         <v>8.13</v>
       </c>
@@ -10604,8 +10636,12 @@
       <c r="C68" t="n">
         <v>0.069</v>
       </c>
-      <c r="D68"/>
-      <c r="E68"/>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
       <c r="F68" t="n">
         <v>10.89</v>
       </c>
@@ -10676,8 +10712,12 @@
       <c r="C70" t="n">
         <v>0.095</v>
       </c>
-      <c r="D70"/>
-      <c r="E70"/>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
       <c r="F70"/>
       <c r="G70"/>
       <c r="H70"/>
@@ -10834,8 +10874,12 @@
       <c r="C75" t="n">
         <v>0.103</v>
       </c>
-      <c r="D75"/>
-      <c r="E75"/>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
       <c r="F75" t="n">
         <v>7.31</v>
       </c>
@@ -11400,8 +11444,12 @@
       <c r="C90" t="n">
         <v>0.174</v>
       </c>
-      <c r="D90"/>
-      <c r="E90"/>
+      <c r="D90" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0</v>
+      </c>
       <c r="F90" t="n">
         <v>7.58</v>
       </c>
@@ -11472,8 +11520,12 @@
       <c r="C92" t="n">
         <v>0.041</v>
       </c>
-      <c r="D92"/>
-      <c r="E92"/>
+      <c r="D92" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" t="n">
+        <v>0</v>
+      </c>
       <c r="F92" t="n">
         <v>6.21</v>
       </c>
@@ -11582,8 +11634,12 @@
       <c r="C95" t="n">
         <v>0.097</v>
       </c>
-      <c r="D95"/>
-      <c r="E95"/>
+      <c r="D95" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" t="n">
+        <v>0</v>
+      </c>
       <c r="F95" t="n">
         <v>11.59</v>
       </c>
@@ -11768,8 +11824,12 @@
       <c r="C100" t="n">
         <v>0.118</v>
       </c>
-      <c r="D100"/>
-      <c r="E100"/>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" t="n">
+        <v>0</v>
+      </c>
       <c r="F100" t="n">
         <v>7.81</v>
       </c>
@@ -11840,8 +11900,12 @@
       <c r="C102" t="n">
         <v>0.097</v>
       </c>
-      <c r="D102"/>
-      <c r="E102"/>
+      <c r="D102" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" t="n">
+        <v>0</v>
+      </c>
       <c r="F102" t="n">
         <v>9.01</v>
       </c>
@@ -12202,8 +12266,12 @@
       <c r="C112" t="n">
         <v>0.092</v>
       </c>
-      <c r="D112"/>
-      <c r="E112"/>
+      <c r="D112" t="n">
+        <v>0</v>
+      </c>
+      <c r="E112" t="n">
+        <v>0</v>
+      </c>
       <c r="F112" t="n">
         <v>6.27</v>
       </c>
@@ -13034,8 +13102,12 @@
       <c r="C134" t="n">
         <v>0.081</v>
       </c>
-      <c r="D134"/>
-      <c r="E134"/>
+      <c r="D134" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" t="n">
+        <v>0</v>
+      </c>
       <c r="F134" t="n">
         <v>6.94</v>
       </c>
@@ -13068,8 +13140,12 @@
       <c r="C135" t="n">
         <v>0.089</v>
       </c>
-      <c r="D135"/>
-      <c r="E135"/>
+      <c r="D135" t="n">
+        <v>0</v>
+      </c>
+      <c r="E135" t="n">
+        <v>0</v>
+      </c>
       <c r="F135" t="n">
         <v>7.63</v>
       </c>
@@ -13392,8 +13468,12 @@
       <c r="C144" t="n">
         <v>0.071</v>
       </c>
-      <c r="D144"/>
-      <c r="E144"/>
+      <c r="D144" t="n">
+        <v>0</v>
+      </c>
+      <c r="E144" t="n">
+        <v>0</v>
+      </c>
       <c r="F144" t="n">
         <v>7.08</v>
       </c>
@@ -13920,8 +14000,12 @@
       <c r="C158" t="n">
         <v>0.053</v>
       </c>
-      <c r="D158"/>
-      <c r="E158"/>
+      <c r="D158" t="n">
+        <v>0</v>
+      </c>
+      <c r="E158" t="n">
+        <v>0</v>
+      </c>
       <c r="F158" t="n">
         <v>7.26</v>
       </c>
@@ -13992,8 +14076,12 @@
       <c r="C160" t="n">
         <v>0.072</v>
       </c>
-      <c r="D160"/>
-      <c r="E160"/>
+      <c r="D160" t="n">
+        <v>0</v>
+      </c>
+      <c r="E160" t="n">
+        <v>0</v>
+      </c>
       <c r="F160" t="n">
         <v>7.5</v>
       </c>
@@ -14026,8 +14114,12 @@
       <c r="C161" t="n">
         <v>0.075</v>
       </c>
-      <c r="D161"/>
-      <c r="E161"/>
+      <c r="D161" t="n">
+        <v>0</v>
+      </c>
+      <c r="E161" t="n">
+        <v>0</v>
+      </c>
       <c r="F161" t="n">
         <v>6.57</v>
       </c>
@@ -14326,8 +14418,12 @@
       <c r="C169" t="n">
         <v>0.078</v>
       </c>
-      <c r="D169"/>
-      <c r="E169"/>
+      <c r="D169" t="n">
+        <v>0</v>
+      </c>
+      <c r="E169" t="n">
+        <v>0</v>
+      </c>
       <c r="F169" t="n">
         <v>7.47</v>
       </c>
@@ -14398,8 +14494,12 @@
       <c r="C171" t="n">
         <v>0.084</v>
       </c>
-      <c r="D171"/>
-      <c r="E171"/>
+      <c r="D171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E171" t="n">
+        <v>0</v>
+      </c>
       <c r="F171" t="n">
         <v>10.81</v>
       </c>
@@ -14622,8 +14722,12 @@
       <c r="C177" t="n">
         <v>0.145</v>
       </c>
-      <c r="D177"/>
-      <c r="E177"/>
+      <c r="D177" t="n">
+        <v>0</v>
+      </c>
+      <c r="E177" t="n">
+        <v>0</v>
+      </c>
       <c r="F177"/>
       <c r="G177"/>
       <c r="H177"/>
@@ -14642,8 +14746,12 @@
       <c r="C178" t="n">
         <v>0.038</v>
       </c>
-      <c r="D178"/>
-      <c r="E178"/>
+      <c r="D178" t="n">
+        <v>0</v>
+      </c>
+      <c r="E178" t="n">
+        <v>0</v>
+      </c>
       <c r="F178" t="n">
         <v>9.39</v>
       </c>
@@ -14928,8 +15036,12 @@
       <c r="C186" t="n">
         <v>0.088</v>
       </c>
-      <c r="D186"/>
-      <c r="E186"/>
+      <c r="D186" t="n">
+        <v>0</v>
+      </c>
+      <c r="E186" t="n">
+        <v>0</v>
+      </c>
       <c r="F186" t="n">
         <v>4.62</v>
       </c>
@@ -15228,8 +15340,12 @@
       <c r="C194" t="n">
         <v>0.099</v>
       </c>
-      <c r="D194"/>
-      <c r="E194"/>
+      <c r="D194" t="n">
+        <v>0</v>
+      </c>
+      <c r="E194" t="n">
+        <v>0</v>
+      </c>
       <c r="F194" t="n">
         <v>3.66</v>
       </c>
@@ -15262,8 +15378,12 @@
       <c r="C195" t="n">
         <v>0.104</v>
       </c>
-      <c r="D195"/>
-      <c r="E195"/>
+      <c r="D195" t="n">
+        <v>0</v>
+      </c>
+      <c r="E195" t="n">
+        <v>0</v>
+      </c>
       <c r="F195" t="n">
         <v>5.26</v>
       </c>
@@ -15334,8 +15454,12 @@
       <c r="C197" t="n">
         <v>0.209</v>
       </c>
-      <c r="D197"/>
-      <c r="E197"/>
+      <c r="D197" t="n">
+        <v>0</v>
+      </c>
+      <c r="E197" t="n">
+        <v>0</v>
+      </c>
       <c r="F197" t="n">
         <v>6.67</v>
       </c>
@@ -15406,8 +15530,12 @@
       <c r="C199" t="n">
         <v>0.155</v>
       </c>
-      <c r="D199"/>
-      <c r="E199"/>
+      <c r="D199" t="n">
+        <v>0</v>
+      </c>
+      <c r="E199" t="n">
+        <v>0</v>
+      </c>
       <c r="F199" t="n">
         <v>3.6</v>
       </c>
@@ -15440,8 +15568,12 @@
       <c r="C200" t="n">
         <v>0.13</v>
       </c>
-      <c r="D200"/>
-      <c r="E200"/>
+      <c r="D200" t="n">
+        <v>0</v>
+      </c>
+      <c r="E200" t="n">
+        <v>0</v>
+      </c>
       <c r="F200" t="n">
         <v>6.68</v>
       </c>
@@ -15550,8 +15682,12 @@
       <c r="C203" t="n">
         <v>0.226</v>
       </c>
-      <c r="D203"/>
-      <c r="E203"/>
+      <c r="D203" t="n">
+        <v>0</v>
+      </c>
+      <c r="E203" t="n">
+        <v>0</v>
+      </c>
       <c r="F203" t="n">
         <v>13.04</v>
       </c>
@@ -15584,8 +15720,12 @@
       <c r="C204" t="n">
         <v>0.185</v>
       </c>
-      <c r="D204"/>
-      <c r="E204"/>
+      <c r="D204" t="n">
+        <v>0</v>
+      </c>
+      <c r="E204" t="n">
+        <v>0</v>
+      </c>
       <c r="F204" t="n">
         <v>9.81</v>
       </c>
@@ -15808,8 +15948,12 @@
       <c r="C210" t="n">
         <v>0.063</v>
       </c>
-      <c r="D210"/>
-      <c r="E210"/>
+      <c r="D210" t="n">
+        <v>0</v>
+      </c>
+      <c r="E210" t="n">
+        <v>0</v>
+      </c>
       <c r="F210" t="n">
         <v>8.53</v>
       </c>
@@ -16070,8 +16214,12 @@
       <c r="C217" t="n">
         <v>0.092</v>
       </c>
-      <c r="D217"/>
-      <c r="E217"/>
+      <c r="D217" t="n">
+        <v>0</v>
+      </c>
+      <c r="E217" t="n">
+        <v>0</v>
+      </c>
       <c r="F217"/>
       <c r="G217"/>
       <c r="H217"/>
@@ -16166,8 +16314,12 @@
       <c r="C220" t="n">
         <v>0.117</v>
       </c>
-      <c r="D220"/>
-      <c r="E220"/>
+      <c r="D220" t="n">
+        <v>0</v>
+      </c>
+      <c r="E220" t="n">
+        <v>0</v>
+      </c>
       <c r="F220" t="n">
         <v>6.82</v>
       </c>
@@ -18314,8 +18466,12 @@
       <c r="C277" t="n">
         <v>0.047</v>
       </c>
-      <c r="D277"/>
-      <c r="E277"/>
+      <c r="D277" t="n">
+        <v>0</v>
+      </c>
+      <c r="E277" t="n">
+        <v>0</v>
+      </c>
       <c r="F277" t="n">
         <v>8.42</v>
       </c>
@@ -18424,8 +18580,12 @@
       <c r="C280" t="n">
         <v>0.073</v>
       </c>
-      <c r="D280"/>
-      <c r="E280"/>
+      <c r="D280" t="n">
+        <v>0</v>
+      </c>
+      <c r="E280" t="n">
+        <v>0</v>
+      </c>
       <c r="F280" t="n">
         <v>10.76</v>
       </c>
@@ -19142,8 +19302,12 @@
       <c r="C299" t="n">
         <v>0.068</v>
       </c>
-      <c r="D299"/>
-      <c r="E299"/>
+      <c r="D299" t="n">
+        <v>0</v>
+      </c>
+      <c r="E299" t="n">
+        <v>0</v>
+      </c>
       <c r="F299" t="n">
         <v>11.55</v>
       </c>
@@ -19480,8 +19644,12 @@
       <c r="C308" t="n">
         <v>0.039</v>
       </c>
-      <c r="D308"/>
-      <c r="E308"/>
+      <c r="D308" t="n">
+        <v>0</v>
+      </c>
+      <c r="E308" t="n">
+        <v>0</v>
+      </c>
       <c r="F308" t="n">
         <v>6.6</v>
       </c>
@@ -19894,8 +20062,12 @@
       <c r="C319" t="n">
         <v>0.019</v>
       </c>
-      <c r="D319"/>
-      <c r="E319"/>
+      <c r="D319" t="n">
+        <v>0</v>
+      </c>
+      <c r="E319" t="n">
+        <v>0</v>
+      </c>
       <c r="F319" t="n">
         <v>12.67</v>
       </c>
@@ -19928,8 +20100,12 @@
       <c r="C320" t="n">
         <v>0.054</v>
       </c>
-      <c r="D320"/>
-      <c r="E320"/>
+      <c r="D320" t="n">
+        <v>0</v>
+      </c>
+      <c r="E320" t="n">
+        <v>0</v>
+      </c>
       <c r="F320" t="n">
         <v>7.62</v>
       </c>
@@ -20000,8 +20176,12 @@
       <c r="C322" t="n">
         <v>0.044</v>
       </c>
-      <c r="D322"/>
-      <c r="E322"/>
+      <c r="D322" t="n">
+        <v>0</v>
+      </c>
+      <c r="E322" t="n">
+        <v>0</v>
+      </c>
       <c r="F322" t="n">
         <v>12.08</v>
       </c>
@@ -20034,8 +20214,12 @@
       <c r="C323" t="n">
         <v>0.022</v>
       </c>
-      <c r="D323"/>
-      <c r="E323"/>
+      <c r="D323" t="n">
+        <v>0</v>
+      </c>
+      <c r="E323" t="n">
+        <v>0</v>
+      </c>
       <c r="F323" t="n">
         <v>6.71</v>
       </c>
@@ -20258,8 +20442,12 @@
       <c r="C329" t="n">
         <v>0.037</v>
       </c>
-      <c r="D329"/>
-      <c r="E329"/>
+      <c r="D329" t="n">
+        <v>0</v>
+      </c>
+      <c r="E329" t="n">
+        <v>0</v>
+      </c>
       <c r="F329" t="n">
         <v>8.06</v>
       </c>
@@ -21114,8 +21302,12 @@
       <c r="C352" t="n">
         <v>0.027</v>
       </c>
-      <c r="D352"/>
-      <c r="E352"/>
+      <c r="D352" t="n">
+        <v>0</v>
+      </c>
+      <c r="E352" t="n">
+        <v>0</v>
+      </c>
       <c r="F352" t="n">
         <v>6.64</v>
       </c>
@@ -21794,8 +21986,12 @@
       <c r="C370" t="n">
         <v>0.056</v>
       </c>
-      <c r="D370"/>
-      <c r="E370"/>
+      <c r="D370" t="n">
+        <v>0</v>
+      </c>
+      <c r="E370" t="n">
+        <v>0</v>
+      </c>
       <c r="F370" t="n">
         <v>9.33</v>
       </c>
@@ -23752,8 +23948,12 @@
       <c r="C422" t="n">
         <v>0.053</v>
       </c>
-      <c r="D422"/>
-      <c r="E422"/>
+      <c r="D422" t="n">
+        <v>0</v>
+      </c>
+      <c r="E422" t="n">
+        <v>0</v>
+      </c>
       <c r="F422" t="n">
         <v>7.44</v>
       </c>
@@ -23900,8 +24100,12 @@
       <c r="C426" t="n">
         <v>0.044</v>
       </c>
-      <c r="D426"/>
-      <c r="E426"/>
+      <c r="D426" t="n">
+        <v>0</v>
+      </c>
+      <c r="E426" t="n">
+        <v>0</v>
+      </c>
       <c r="F426" t="n">
         <v>7.84</v>
       </c>
@@ -23934,8 +24138,12 @@
       <c r="C427" t="n">
         <v>0.013</v>
       </c>
-      <c r="D427"/>
-      <c r="E427"/>
+      <c r="D427" t="n">
+        <v>0</v>
+      </c>
+      <c r="E427" t="n">
+        <v>0</v>
+      </c>
       <c r="F427" t="n">
         <v>8.21</v>
       </c>
@@ -24310,8 +24518,12 @@
       <c r="C437" t="n">
         <v>0.079</v>
       </c>
-      <c r="D437"/>
-      <c r="E437"/>
+      <c r="D437" t="n">
+        <v>0</v>
+      </c>
+      <c r="E437" t="n">
+        <v>0</v>
+      </c>
       <c r="F437" t="n">
         <v>7.51</v>
       </c>
@@ -24420,8 +24632,12 @@
       <c r="C440" t="n">
         <v>0.005</v>
       </c>
-      <c r="D440"/>
-      <c r="E440"/>
+      <c r="D440" t="n">
+        <v>0</v>
+      </c>
+      <c r="E440" t="n">
+        <v>0</v>
+      </c>
       <c r="F440" t="n">
         <v>7.9</v>
       </c>
@@ -25062,8 +25278,12 @@
       <c r="C457" t="n">
         <v>0.051</v>
       </c>
-      <c r="D457"/>
-      <c r="E457"/>
+      <c r="D457" t="n">
+        <v>0</v>
+      </c>
+      <c r="E457" t="n">
+        <v>0</v>
+      </c>
       <c r="F457" t="n">
         <v>6.76</v>
       </c>
@@ -26004,8 +26224,12 @@
       <c r="C483" t="n">
         <v>0.093</v>
       </c>
-      <c r="D483"/>
-      <c r="E483"/>
+      <c r="D483" t="n">
+        <v>0</v>
+      </c>
+      <c r="E483" t="n">
+        <v>0</v>
+      </c>
       <c r="F483" t="n">
         <v>8.45</v>
       </c>
@@ -26038,8 +26262,12 @@
       <c r="C484" t="n">
         <v>0.043</v>
       </c>
-      <c r="D484"/>
-      <c r="E484"/>
+      <c r="D484" t="n">
+        <v>0</v>
+      </c>
+      <c r="E484" t="n">
+        <v>0</v>
+      </c>
       <c r="F484" t="n">
         <v>6.61</v>
       </c>
@@ -26338,8 +26566,12 @@
       <c r="C492" t="n">
         <v>0.071</v>
       </c>
-      <c r="D492"/>
-      <c r="E492"/>
+      <c r="D492" t="n">
+        <v>0</v>
+      </c>
+      <c r="E492" t="n">
+        <v>0</v>
+      </c>
       <c r="F492" t="n">
         <v>9.59</v>
       </c>
@@ -26372,8 +26604,12 @@
       <c r="C493" t="n">
         <v>0.046</v>
       </c>
-      <c r="D493"/>
-      <c r="E493"/>
+      <c r="D493" t="n">
+        <v>0</v>
+      </c>
+      <c r="E493" t="n">
+        <v>0</v>
+      </c>
       <c r="F493" t="n">
         <v>8.11</v>
       </c>
@@ -26406,8 +26642,12 @@
       <c r="C494" t="n">
         <v>0.058</v>
       </c>
-      <c r="D494"/>
-      <c r="E494"/>
+      <c r="D494" t="n">
+        <v>0</v>
+      </c>
+      <c r="E494" t="n">
+        <v>0</v>
+      </c>
       <c r="F494" t="n">
         <v>7.44</v>
       </c>
@@ -26554,8 +26794,12 @@
       <c r="C498" t="n">
         <v>0.067</v>
       </c>
-      <c r="D498"/>
-      <c r="E498"/>
+      <c r="D498" t="n">
+        <v>0</v>
+      </c>
+      <c r="E498" t="n">
+        <v>0</v>
+      </c>
       <c r="F498" t="n">
         <v>6.38</v>
       </c>
@@ -26992,8 +27236,12 @@
       <c r="C510" t="n">
         <v>0.099</v>
       </c>
-      <c r="D510"/>
-      <c r="E510"/>
+      <c r="D510" t="n">
+        <v>0</v>
+      </c>
+      <c r="E510" t="n">
+        <v>0</v>
+      </c>
       <c r="F510" t="n">
         <v>8.97</v>
       </c>
@@ -27026,8 +27274,12 @@
       <c r="C511" t="n">
         <v>0.054</v>
       </c>
-      <c r="D511"/>
-      <c r="E511"/>
+      <c r="D511" t="n">
+        <v>0</v>
+      </c>
+      <c r="E511" t="n">
+        <v>0</v>
+      </c>
       <c r="F511" t="n">
         <v>7.33</v>
       </c>
@@ -27060,8 +27312,12 @@
       <c r="C512" t="n">
         <v>0.027</v>
       </c>
-      <c r="D512"/>
-      <c r="E512"/>
+      <c r="D512" t="n">
+        <v>0</v>
+      </c>
+      <c r="E512" t="n">
+        <v>0</v>
+      </c>
       <c r="F512" t="n">
         <v>7.54</v>
       </c>
@@ -27722,8 +27978,12 @@
       <c r="C531" t="n">
         <v>0.093</v>
       </c>
-      <c r="D531"/>
-      <c r="E531"/>
+      <c r="D531" t="n">
+        <v>0</v>
+      </c>
+      <c r="E531" t="n">
+        <v>0</v>
+      </c>
       <c r="F531" t="n">
         <v>8.01</v>
       </c>
@@ -27794,8 +28054,12 @@
       <c r="C533" t="n">
         <v>0.072</v>
       </c>
-      <c r="D533"/>
-      <c r="E533"/>
+      <c r="D533" t="n">
+        <v>0</v>
+      </c>
+      <c r="E533" t="n">
+        <v>0</v>
+      </c>
       <c r="F533" t="n">
         <v>5.92</v>
       </c>
@@ -27866,8 +28130,12 @@
       <c r="C535" t="n">
         <v>0.032</v>
       </c>
-      <c r="D535"/>
-      <c r="E535"/>
+      <c r="D535" t="n">
+        <v>0</v>
+      </c>
+      <c r="E535" t="n">
+        <v>0</v>
+      </c>
       <c r="F535" t="n">
         <v>6.47</v>
       </c>
@@ -27900,8 +28168,12 @@
       <c r="C536" t="n">
         <v>0.055</v>
       </c>
-      <c r="D536"/>
-      <c r="E536"/>
+      <c r="D536" t="n">
+        <v>0</v>
+      </c>
+      <c r="E536" t="n">
+        <v>0</v>
+      </c>
       <c r="F536" t="n">
         <v>9.21</v>
       </c>
@@ -28238,8 +28510,12 @@
       <c r="C545" t="n">
         <v>0.083</v>
       </c>
-      <c r="D545"/>
-      <c r="E545"/>
+      <c r="D545" t="n">
+        <v>0</v>
+      </c>
+      <c r="E545" t="n">
+        <v>0</v>
+      </c>
       <c r="F545" t="n">
         <v>11.64</v>
       </c>
@@ -28386,8 +28662,12 @@
       <c r="C549" t="n">
         <v>0.034</v>
       </c>
-      <c r="D549"/>
-      <c r="E549"/>
+      <c r="D549" t="n">
+        <v>0</v>
+      </c>
+      <c r="E549" t="n">
+        <v>0</v>
+      </c>
       <c r="F549" t="n">
         <v>8.43</v>
       </c>
@@ -28990,8 +29270,12 @@
       <c r="C565" t="n">
         <v>0.031</v>
       </c>
-      <c r="D565"/>
-      <c r="E565"/>
+      <c r="D565" t="n">
+        <v>0</v>
+      </c>
+      <c r="E565" t="n">
+        <v>0</v>
+      </c>
       <c r="F565" t="n">
         <v>7.09</v>
       </c>
@@ -29404,8 +29688,12 @@
       <c r="C576" t="n">
         <v>0.018</v>
       </c>
-      <c r="D576"/>
-      <c r="E576"/>
+      <c r="D576" t="n">
+        <v>0</v>
+      </c>
+      <c r="E576" t="n">
+        <v>0</v>
+      </c>
       <c r="F576" t="n">
         <v>11.48</v>
       </c>
@@ -29438,8 +29726,12 @@
       <c r="C577" t="n">
         <v>0.056</v>
       </c>
-      <c r="D577"/>
-      <c r="E577"/>
+      <c r="D577" t="n">
+        <v>0</v>
+      </c>
+      <c r="E577" t="n">
+        <v>0</v>
+      </c>
       <c r="F577" t="n">
         <v>6.47</v>
       </c>
@@ -29548,8 +29840,12 @@
       <c r="C580" t="n">
         <v>0.044</v>
       </c>
-      <c r="D580"/>
-      <c r="E580"/>
+      <c r="D580" t="n">
+        <v>0</v>
+      </c>
+      <c r="E580" t="n">
+        <v>0</v>
+      </c>
       <c r="F580" t="n">
         <v>7.42</v>
       </c>
@@ -29582,8 +29878,12 @@
       <c r="C581" t="n">
         <v>0.025</v>
       </c>
-      <c r="D581"/>
-      <c r="E581"/>
+      <c r="D581" t="n">
+        <v>0</v>
+      </c>
+      <c r="E581" t="n">
+        <v>0</v>
+      </c>
       <c r="F581" t="n">
         <v>6.94</v>
       </c>
@@ -30058,8 +30358,12 @@
       <c r="C594" t="n">
         <v>0.092</v>
       </c>
-      <c r="D594"/>
-      <c r="E594"/>
+      <c r="D594" t="n">
+        <v>0</v>
+      </c>
+      <c r="E594" t="n">
+        <v>0</v>
+      </c>
       <c r="F594" t="n">
         <v>7.1</v>
       </c>
@@ -30168,8 +30472,12 @@
       <c r="C597" t="n">
         <v>0.136</v>
       </c>
-      <c r="D597"/>
-      <c r="E597"/>
+      <c r="D597" t="n">
+        <v>0</v>
+      </c>
+      <c r="E597" t="n">
+        <v>0</v>
+      </c>
       <c r="F597" t="n">
         <v>7.47</v>
       </c>
@@ -30202,8 +30510,12 @@
       <c r="C598" t="n">
         <v>0.044</v>
       </c>
-      <c r="D598"/>
-      <c r="E598"/>
+      <c r="D598" t="n">
+        <v>0</v>
+      </c>
+      <c r="E598" t="n">
+        <v>0</v>
+      </c>
       <c r="F598" t="n">
         <v>7.49</v>
       </c>
@@ -30236,8 +30548,12 @@
       <c r="C599" t="n">
         <v>0.08</v>
       </c>
-      <c r="D599"/>
-      <c r="E599"/>
+      <c r="D599" t="n">
+        <v>0</v>
+      </c>
+      <c r="E599" t="n">
+        <v>0</v>
+      </c>
       <c r="F599" t="n">
         <v>2.81</v>
       </c>
@@ -30308,8 +30624,12 @@
       <c r="C601" t="n">
         <v>0.073</v>
       </c>
-      <c r="D601"/>
-      <c r="E601"/>
+      <c r="D601" t="n">
+        <v>0</v>
+      </c>
+      <c r="E601" t="n">
+        <v>0</v>
+      </c>
       <c r="F601" t="n">
         <v>4.23</v>
       </c>
@@ -30380,8 +30700,12 @@
       <c r="C603" t="n">
         <v>0.06</v>
       </c>
-      <c r="D603"/>
-      <c r="E603"/>
+      <c r="D603" t="n">
+        <v>0</v>
+      </c>
+      <c r="E603" t="n">
+        <v>0</v>
+      </c>
       <c r="F603" t="n">
         <v>4.47</v>
       </c>
@@ -30894,8 +31218,12 @@
       <c r="C617" t="n">
         <v>0.075</v>
       </c>
-      <c r="D617"/>
-      <c r="E617"/>
+      <c r="D617" t="n">
+        <v>0</v>
+      </c>
+      <c r="E617" t="n">
+        <v>0</v>
+      </c>
       <c r="F617" t="n">
         <v>17.35</v>
       </c>
@@ -31004,8 +31332,12 @@
       <c r="C620" t="n">
         <v>0.109</v>
       </c>
-      <c r="D620"/>
-      <c r="E620"/>
+      <c r="D620" t="n">
+        <v>0</v>
+      </c>
+      <c r="E620" t="n">
+        <v>0</v>
+      </c>
       <c r="F620" t="n">
         <v>7.07</v>
       </c>
@@ -31076,8 +31408,12 @@
       <c r="C622" t="n">
         <v>0.107</v>
       </c>
-      <c r="D622"/>
-      <c r="E622"/>
+      <c r="D622" t="n">
+        <v>0</v>
+      </c>
+      <c r="E622" t="n">
+        <v>0</v>
+      </c>
       <c r="F622" t="n">
         <v>7.12</v>
       </c>
@@ -31186,8 +31522,12 @@
       <c r="C625" t="n">
         <v>0.065</v>
       </c>
-      <c r="D625"/>
-      <c r="E625"/>
+      <c r="D625" t="n">
+        <v>0</v>
+      </c>
+      <c r="E625" t="n">
+        <v>0</v>
+      </c>
       <c r="F625" t="n">
         <v>8.27</v>
       </c>
@@ -31258,8 +31598,12 @@
       <c r="C627" t="n">
         <v>0.094</v>
       </c>
-      <c r="D627"/>
-      <c r="E627"/>
+      <c r="D627" t="n">
+        <v>0</v>
+      </c>
+      <c r="E627" t="n">
+        <v>0</v>
+      </c>
       <c r="F627" t="n">
         <v>9.58</v>
       </c>
@@ -31672,8 +32016,12 @@
       <c r="C638" t="n">
         <v>0.063</v>
       </c>
-      <c r="D638"/>
-      <c r="E638"/>
+      <c r="D638" t="n">
+        <v>0</v>
+      </c>
+      <c r="E638" t="n">
+        <v>0</v>
+      </c>
       <c r="F638" t="n">
         <v>2.59</v>
       </c>
@@ -31782,8 +32130,12 @@
       <c r="C641" t="n">
         <v>0.128</v>
       </c>
-      <c r="D641"/>
-      <c r="E641"/>
+      <c r="D641" t="n">
+        <v>0</v>
+      </c>
+      <c r="E641" t="n">
+        <v>0</v>
+      </c>
       <c r="F641" t="n">
         <v>7.15</v>
       </c>
@@ -32310,8 +32662,12 @@
       <c r="C655" t="n">
         <v>0.063</v>
       </c>
-      <c r="D655"/>
-      <c r="E655"/>
+      <c r="D655" t="n">
+        <v>0</v>
+      </c>
+      <c r="E655" t="n">
+        <v>0</v>
+      </c>
       <c r="F655" t="n">
         <v>6.46</v>
       </c>
@@ -32344,8 +32700,12 @@
       <c r="C656" t="n">
         <v>0.072</v>
       </c>
-      <c r="D656"/>
-      <c r="E656"/>
+      <c r="D656" t="n">
+        <v>0</v>
+      </c>
+      <c r="E656" t="n">
+        <v>0</v>
+      </c>
       <c r="F656" t="n">
         <v>6.08</v>
       </c>
@@ -32416,8 +32776,12 @@
       <c r="C658" t="n">
         <v>0.047</v>
       </c>
-      <c r="D658"/>
-      <c r="E658"/>
+      <c r="D658" t="n">
+        <v>0</v>
+      </c>
+      <c r="E658" t="n">
+        <v>0</v>
+      </c>
       <c r="F658" t="n">
         <v>7.82</v>
       </c>
@@ -32640,8 +33004,12 @@
       <c r="C664" t="n">
         <v>0.066</v>
       </c>
-      <c r="D664"/>
-      <c r="E664"/>
+      <c r="D664" t="n">
+        <v>0</v>
+      </c>
+      <c r="E664" t="n">
+        <v>0</v>
+      </c>
       <c r="F664" t="n">
         <v>19.44</v>
       </c>
@@ -32750,8 +33118,12 @@
       <c r="C667" t="n">
         <v>0.06</v>
       </c>
-      <c r="D667"/>
-      <c r="E667"/>
+      <c r="D667" t="n">
+        <v>0</v>
+      </c>
+      <c r="E667" t="n">
+        <v>0</v>
+      </c>
       <c r="F667" t="n">
         <v>7.47</v>
       </c>
@@ -32784,8 +33156,12 @@
       <c r="C668" t="n">
         <v>0.07</v>
       </c>
-      <c r="D668"/>
-      <c r="E668"/>
+      <c r="D668" t="n">
+        <v>0</v>
+      </c>
+      <c r="E668" t="n">
+        <v>0</v>
+      </c>
       <c r="F668" t="n">
         <v>6.71</v>
       </c>
@@ -33312,8 +33688,12 @@
       <c r="C682" t="n">
         <v>0.062</v>
       </c>
-      <c r="D682"/>
-      <c r="E682"/>
+      <c r="D682" t="n">
+        <v>0</v>
+      </c>
+      <c r="E682" t="n">
+        <v>0</v>
+      </c>
       <c r="F682" t="n">
         <v>6.09</v>
       </c>
@@ -33726,8 +34106,12 @@
       <c r="C693" t="n">
         <v>0.017</v>
       </c>
-      <c r="D693"/>
-      <c r="E693"/>
+      <c r="D693" t="n">
+        <v>0</v>
+      </c>
+      <c r="E693" t="n">
+        <v>0</v>
+      </c>
       <c r="F693"/>
       <c r="G693"/>
       <c r="H693"/>
@@ -33936,8 +34320,12 @@
       <c r="C699" t="n">
         <v>0.007</v>
       </c>
-      <c r="D699"/>
-      <c r="E699"/>
+      <c r="D699" t="n">
+        <v>0</v>
+      </c>
+      <c r="E699" t="n">
+        <v>0</v>
+      </c>
       <c r="F699"/>
       <c r="G699"/>
       <c r="H699"/>
@@ -33991,7 +34379,9 @@
       <c r="B701" t="n">
         <v>94.374</v>
       </c>
-      <c r="C701"/>
+      <c r="C701" t="n">
+        <v>0</v>
+      </c>
       <c r="D701" t="n">
         <v>52.5</v>
       </c>
@@ -34548,8 +34938,12 @@
       <c r="C716" t="n">
         <v>0</v>
       </c>
-      <c r="D716"/>
-      <c r="E716"/>
+      <c r="D716" t="n">
+        <v>0</v>
+      </c>
+      <c r="E716" t="n">
+        <v>0</v>
+      </c>
       <c r="F716" t="n">
         <v>8.75</v>
       </c>
@@ -34962,8 +35356,12 @@
       <c r="C727" t="n">
         <v>0.012</v>
       </c>
-      <c r="D727"/>
-      <c r="E727"/>
+      <c r="D727" t="n">
+        <v>0</v>
+      </c>
+      <c r="E727" t="n">
+        <v>0</v>
+      </c>
       <c r="F727" t="n">
         <v>9.31</v>
       </c>
@@ -37148,8 +37546,12 @@
       <c r="C785" t="n">
         <v>0.002</v>
       </c>
-      <c r="D785"/>
-      <c r="E785"/>
+      <c r="D785" t="n">
+        <v>0</v>
+      </c>
+      <c r="E785" t="n">
+        <v>0</v>
+      </c>
       <c r="F785" t="n">
         <v>8.13</v>
       </c>
@@ -37179,7 +37581,9 @@
       <c r="B786" t="n">
         <v>92.166</v>
       </c>
-      <c r="C786"/>
+      <c r="C786" t="n">
+        <v>0</v>
+      </c>
       <c r="D786" t="n">
         <v>149.4</v>
       </c>
@@ -37294,8 +37698,12 @@
       <c r="C789" t="n">
         <v>0.004</v>
       </c>
-      <c r="D789"/>
-      <c r="E789"/>
+      <c r="D789" t="n">
+        <v>0</v>
+      </c>
+      <c r="E789" t="n">
+        <v>0</v>
+      </c>
       <c r="F789" t="n">
         <v>8.62</v>
       </c>
@@ -37708,8 +38116,12 @@
       <c r="C800" t="n">
         <v>0.072</v>
       </c>
-      <c r="D800"/>
-      <c r="E800"/>
+      <c r="D800" t="n">
+        <v>0</v>
+      </c>
+      <c r="E800" t="n">
+        <v>0</v>
+      </c>
       <c r="F800" t="n">
         <v>8.08</v>
       </c>
@@ -37818,8 +38230,12 @@
       <c r="C803" t="n">
         <v>0.013</v>
       </c>
-      <c r="D803"/>
-      <c r="E803"/>
+      <c r="D803" t="n">
+        <v>0</v>
+      </c>
+      <c r="E803" t="n">
+        <v>0</v>
+      </c>
       <c r="F803" t="n">
         <v>8.52</v>
       </c>
@@ -38232,8 +38648,12 @@
       <c r="C814" t="n">
         <v>0.006</v>
       </c>
-      <c r="D814"/>
-      <c r="E814"/>
+      <c r="D814" t="n">
+        <v>0</v>
+      </c>
+      <c r="E814" t="n">
+        <v>0</v>
+      </c>
       <c r="F814" t="n">
         <v>7.88</v>
       </c>
@@ -39112,8 +39532,12 @@
       <c r="C838" t="n">
         <v>0.096</v>
       </c>
-      <c r="D838"/>
-      <c r="E838"/>
+      <c r="D838" t="n">
+        <v>0</v>
+      </c>
+      <c r="E838" t="n">
+        <v>0</v>
+      </c>
       <c r="F838"/>
       <c r="G838"/>
       <c r="H838"/>
@@ -39536,8 +39960,12 @@
       <c r="C850" t="n">
         <v>0.031</v>
       </c>
-      <c r="D850"/>
-      <c r="E850"/>
+      <c r="D850" t="n">
+        <v>0</v>
+      </c>
+      <c r="E850" t="n">
+        <v>0</v>
+      </c>
       <c r="F850" t="n">
         <v>8.38</v>
       </c>
@@ -40254,8 +40682,12 @@
       <c r="C869" t="n">
         <v>0.019</v>
       </c>
-      <c r="D869"/>
-      <c r="E869"/>
+      <c r="D869" t="n">
+        <v>0</v>
+      </c>
+      <c r="E869" t="n">
+        <v>0</v>
+      </c>
       <c r="F869" t="n">
         <v>8.8</v>
       </c>
@@ -40288,8 +40720,12 @@
       <c r="C870" t="n">
         <v>0.013</v>
       </c>
-      <c r="D870"/>
-      <c r="E870"/>
+      <c r="D870" t="n">
+        <v>0</v>
+      </c>
+      <c r="E870" t="n">
+        <v>0</v>
+      </c>
       <c r="F870" t="n">
         <v>6.95</v>
       </c>
@@ -40460,8 +40896,12 @@
       <c r="C875" t="n">
         <v>0.01</v>
       </c>
-      <c r="D875"/>
-      <c r="E875"/>
+      <c r="D875" t="n">
+        <v>0</v>
+      </c>
+      <c r="E875" t="n">
+        <v>0</v>
+      </c>
       <c r="F875" t="n">
         <v>8.79</v>
       </c>
@@ -40532,8 +40972,12 @@
       <c r="C877" t="n">
         <v>0.019</v>
       </c>
-      <c r="D877"/>
-      <c r="E877"/>
+      <c r="D877" t="n">
+        <v>0</v>
+      </c>
+      <c r="E877" t="n">
+        <v>0</v>
+      </c>
       <c r="F877" t="n">
         <v>9</v>
       </c>
@@ -40832,8 +41276,12 @@
       <c r="C885" t="n">
         <v>0.002</v>
       </c>
-      <c r="D885"/>
-      <c r="E885"/>
+      <c r="D885" t="n">
+        <v>0</v>
+      </c>
+      <c r="E885" t="n">
+        <v>0</v>
+      </c>
       <c r="F885" t="n">
         <v>9.58</v>
       </c>
@@ -40866,8 +41314,12 @@
       <c r="C886" t="n">
         <v>0.043</v>
       </c>
-      <c r="D886"/>
-      <c r="E886"/>
+      <c r="D886" t="n">
+        <v>0</v>
+      </c>
+      <c r="E886" t="n">
+        <v>0</v>
+      </c>
       <c r="F886" t="n">
         <v>6.59</v>
       </c>
@@ -41377,7 +41829,9 @@
       <c r="B900" t="n">
         <v>92.043</v>
       </c>
-      <c r="C900"/>
+      <c r="C900" t="n">
+        <v>0</v>
+      </c>
       <c r="D900" t="n">
         <v>468.5</v>
       </c>
@@ -41606,8 +42060,12 @@
       <c r="C906" t="n">
         <v>0.038</v>
       </c>
-      <c r="D906"/>
-      <c r="E906"/>
+      <c r="D906" t="n">
+        <v>0</v>
+      </c>
+      <c r="E906" t="n">
+        <v>0</v>
+      </c>
       <c r="F906" t="n">
         <v>8.1</v>
       </c>
@@ -41830,8 +42288,12 @@
       <c r="C912" t="n">
         <v>0.042</v>
       </c>
-      <c r="D912"/>
-      <c r="E912"/>
+      <c r="D912" t="n">
+        <v>0</v>
+      </c>
+      <c r="E912" t="n">
+        <v>0</v>
+      </c>
       <c r="F912" t="n">
         <v>7.79</v>
       </c>
@@ -41978,8 +42440,12 @@
       <c r="C916" t="n">
         <v>0.012</v>
       </c>
-      <c r="D916"/>
-      <c r="E916"/>
+      <c r="D916" t="n">
+        <v>0</v>
+      </c>
+      <c r="E916" t="n">
+        <v>0</v>
+      </c>
       <c r="F916" t="n">
         <v>8.68</v>
       </c>
@@ -42620,8 +43086,12 @@
       <c r="C933" t="n">
         <v>0.058</v>
       </c>
-      <c r="D933"/>
-      <c r="E933"/>
+      <c r="D933" t="n">
+        <v>0</v>
+      </c>
+      <c r="E933" t="n">
+        <v>0</v>
+      </c>
       <c r="F933" t="n">
         <v>7.66</v>
       </c>
@@ -42692,8 +43162,12 @@
       <c r="C935" t="n">
         <v>0.01</v>
       </c>
-      <c r="D935"/>
-      <c r="E935"/>
+      <c r="D935" t="n">
+        <v>0</v>
+      </c>
+      <c r="E935" t="n">
+        <v>0</v>
+      </c>
       <c r="F935" t="n">
         <v>4.59</v>
       </c>
@@ -43030,8 +43504,12 @@
       <c r="C944" t="n">
         <v>0.043</v>
       </c>
-      <c r="D944"/>
-      <c r="E944"/>
+      <c r="D944" t="n">
+        <v>0</v>
+      </c>
+      <c r="E944" t="n">
+        <v>0</v>
+      </c>
       <c r="F944" t="n">
         <v>9.74</v>
       </c>
@@ -43216,8 +43694,12 @@
       <c r="C949" t="n">
         <v>0.083</v>
       </c>
-      <c r="D949"/>
-      <c r="E949"/>
+      <c r="D949" t="n">
+        <v>0</v>
+      </c>
+      <c r="E949" t="n">
+        <v>0</v>
+      </c>
       <c r="F949" t="n">
         <v>14.04</v>
       </c>
@@ -43250,8 +43732,12 @@
       <c r="C950" t="n">
         <v>0.022</v>
       </c>
-      <c r="D950"/>
-      <c r="E950"/>
+      <c r="D950" t="n">
+        <v>0</v>
+      </c>
+      <c r="E950" t="n">
+        <v>0</v>
+      </c>
       <c r="F950" t="n">
         <v>8.22</v>
       </c>
@@ -44500,8 +44986,12 @@
       <c r="C983" t="n">
         <v>0.036</v>
       </c>
-      <c r="D983"/>
-      <c r="E983"/>
+      <c r="D983" t="n">
+        <v>0</v>
+      </c>
+      <c r="E983" t="n">
+        <v>0</v>
+      </c>
       <c r="F983" t="n">
         <v>7.95</v>
       </c>
@@ -44534,8 +45024,12 @@
       <c r="C984" t="n">
         <v>0.084</v>
       </c>
-      <c r="D984"/>
-      <c r="E984"/>
+      <c r="D984" t="n">
+        <v>0</v>
+      </c>
+      <c r="E984" t="n">
+        <v>0</v>
+      </c>
       <c r="F984" t="n">
         <v>15.32</v>
       </c>
@@ -44948,8 +45442,12 @@
       <c r="C995" t="n">
         <v>0.028</v>
       </c>
-      <c r="D995"/>
-      <c r="E995"/>
+      <c r="D995" t="n">
+        <v>0</v>
+      </c>
+      <c r="E995" t="n">
+        <v>0</v>
+      </c>
       <c r="F995" t="n">
         <v>7.09</v>
       </c>
@@ -45210,8 +45708,12 @@
       <c r="C1002" t="n">
         <v>0.065</v>
       </c>
-      <c r="D1002"/>
-      <c r="E1002"/>
+      <c r="D1002" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1002" t="n">
+        <v>0</v>
+      </c>
       <c r="F1002" t="n">
         <v>6.37</v>
       </c>
@@ -45244,8 +45746,12 @@
       <c r="C1003" t="n">
         <v>0.018</v>
       </c>
-      <c r="D1003"/>
-      <c r="E1003"/>
+      <c r="D1003" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1003" t="n">
+        <v>0</v>
+      </c>
       <c r="F1003" t="n">
         <v>8.05</v>
       </c>
@@ -45278,8 +45784,12 @@
       <c r="C1004" t="n">
         <v>0.053</v>
       </c>
-      <c r="D1004"/>
-      <c r="E1004"/>
+      <c r="D1004" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1004" t="n">
+        <v>0</v>
+      </c>
       <c r="F1004" t="n">
         <v>6.81</v>
       </c>
@@ -45426,8 +45936,12 @@
       <c r="C1008" t="n">
         <v>0.092</v>
       </c>
-      <c r="D1008"/>
-      <c r="E1008"/>
+      <c r="D1008" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1008" t="n">
+        <v>0</v>
+      </c>
       <c r="F1008" t="n">
         <v>7.75</v>
       </c>
@@ -45460,8 +45974,12 @@
       <c r="C1009" t="n">
         <v>0.051</v>
       </c>
-      <c r="D1009"/>
-      <c r="E1009"/>
+      <c r="D1009" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1009" t="n">
+        <v>0</v>
+      </c>
       <c r="F1009" t="n">
         <v>7.03</v>
       </c>
@@ -45570,8 +46088,12 @@
       <c r="C1012" t="n">
         <v>0.017</v>
       </c>
-      <c r="D1012"/>
-      <c r="E1012"/>
+      <c r="D1012" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1012" t="n">
+        <v>0</v>
+      </c>
       <c r="F1012" t="n">
         <v>6.52</v>
       </c>
@@ -45984,8 +46506,12 @@
       <c r="C1023" t="n">
         <v>0.052</v>
       </c>
-      <c r="D1023"/>
-      <c r="E1023"/>
+      <c r="D1023" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1023" t="n">
+        <v>0</v>
+      </c>
       <c r="F1023" t="n">
         <v>6.69</v>
       </c>
@@ -46992,8 +47518,12 @@
       <c r="C1050" t="n">
         <v>0.011</v>
       </c>
-      <c r="D1050"/>
-      <c r="E1050"/>
+      <c r="D1050" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1050" t="n">
+        <v>0</v>
+      </c>
       <c r="F1050" t="n">
         <v>8.47</v>
       </c>
@@ -47064,8 +47594,12 @@
       <c r="C1052" t="n">
         <v>0.126</v>
       </c>
-      <c r="D1052"/>
-      <c r="E1052"/>
+      <c r="D1052" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1052" t="n">
+        <v>0</v>
+      </c>
       <c r="F1052" t="n">
         <v>8.3</v>
       </c>
@@ -47512,8 +48046,12 @@
       <c r="C1065" t="n">
         <v>0.269</v>
       </c>
-      <c r="D1065"/>
-      <c r="E1065"/>
+      <c r="D1065" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1065" t="n">
+        <v>0</v>
+      </c>
       <c r="F1065" t="n">
         <v>4.43</v>
       </c>
@@ -47660,8 +48198,12 @@
       <c r="C1069" t="n">
         <v>0.154</v>
       </c>
-      <c r="D1069"/>
-      <c r="E1069"/>
+      <c r="D1069" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1069" t="n">
+        <v>0</v>
+      </c>
       <c r="F1069" t="n">
         <v>9</v>
       </c>
@@ -47794,8 +48336,12 @@
       <c r="C1073" t="n">
         <v>0.044</v>
       </c>
-      <c r="D1073"/>
-      <c r="E1073"/>
+      <c r="D1073" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1073" t="n">
+        <v>0</v>
+      </c>
       <c r="F1073" t="n">
         <v>8.21</v>
       </c>
@@ -48484,8 +49030,12 @@
       <c r="C1092" t="n">
         <v>0.008</v>
       </c>
-      <c r="D1092"/>
-      <c r="E1092"/>
+      <c r="D1092" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1092" t="n">
+        <v>0</v>
+      </c>
       <c r="F1092" t="n">
         <v>8.17</v>
       </c>
@@ -48708,8 +49258,12 @@
       <c r="C1098" t="n">
         <v>0.07</v>
       </c>
-      <c r="D1098"/>
-      <c r="E1098"/>
+      <c r="D1098" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1098" t="n">
+        <v>0</v>
+      </c>
       <c r="F1098" t="n">
         <v>9.57</v>
       </c>
@@ -49198,8 +49752,12 @@
       <c r="C1111" t="n">
         <v>0.023</v>
       </c>
-      <c r="D1111"/>
-      <c r="E1111"/>
+      <c r="D1111" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1111" t="n">
+        <v>0</v>
+      </c>
       <c r="F1111" t="n">
         <v>8.14</v>
       </c>
@@ -49498,8 +50056,12 @@
       <c r="C1119" t="n">
         <v>0.025</v>
       </c>
-      <c r="D1119"/>
-      <c r="E1119"/>
+      <c r="D1119" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1119" t="n">
+        <v>0</v>
+      </c>
       <c r="F1119" t="n">
         <v>9.03</v>
       </c>
@@ -49760,8 +50322,12 @@
       <c r="C1126" t="n">
         <v>0.04</v>
       </c>
-      <c r="D1126"/>
-      <c r="E1126"/>
+      <c r="D1126" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1126" t="n">
+        <v>0</v>
+      </c>
       <c r="F1126" t="n">
         <v>10.26</v>
       </c>
@@ -50274,8 +50840,12 @@
       <c r="C1140" t="n">
         <v>0.026</v>
       </c>
-      <c r="D1140"/>
-      <c r="E1140"/>
+      <c r="D1140" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1140" t="n">
+        <v>0</v>
+      </c>
       <c r="F1140" t="n">
         <v>20.5</v>
       </c>
@@ -50384,8 +50954,12 @@
       <c r="C1143" t="n">
         <v>0.033</v>
       </c>
-      <c r="D1143"/>
-      <c r="E1143"/>
+      <c r="D1143" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1143" t="n">
+        <v>0</v>
+      </c>
       <c r="F1143" t="n">
         <v>9.91</v>
       </c>
@@ -50746,8 +51320,12 @@
       <c r="C1153" t="n">
         <v>0.025</v>
       </c>
-      <c r="D1153"/>
-      <c r="E1153"/>
+      <c r="D1153" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1153" t="n">
+        <v>0</v>
+      </c>
       <c r="F1153" t="n">
         <v>15.53</v>
       </c>
@@ -50818,8 +51396,12 @@
       <c r="C1155" t="n">
         <v>0.01</v>
       </c>
-      <c r="D1155"/>
-      <c r="E1155"/>
+      <c r="D1155" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1155" t="n">
+        <v>0</v>
+      </c>
       <c r="F1155" t="n">
         <v>18.21</v>
       </c>
@@ -50852,8 +51434,12 @@
       <c r="C1156" t="n">
         <v>0.037</v>
       </c>
-      <c r="D1156"/>
-      <c r="E1156"/>
+      <c r="D1156" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1156" t="n">
+        <v>0</v>
+      </c>
       <c r="F1156" t="n">
         <v>10.95</v>
       </c>
@@ -50886,8 +51472,12 @@
       <c r="C1157" t="n">
         <v>0.027</v>
       </c>
-      <c r="D1157"/>
-      <c r="E1157"/>
+      <c r="D1157" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1157" t="n">
+        <v>0</v>
+      </c>
       <c r="F1157" t="n">
         <v>10.86</v>
       </c>
@@ -51110,8 +51700,12 @@
       <c r="C1163" t="n">
         <v>0.06</v>
       </c>
-      <c r="D1163"/>
-      <c r="E1163"/>
+      <c r="D1163" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1163" t="n">
+        <v>0</v>
+      </c>
       <c r="F1163" t="n">
         <v>6.38</v>
       </c>
@@ -51548,8 +52142,12 @@
       <c r="C1175" t="n">
         <v>0.044</v>
       </c>
-      <c r="D1175"/>
-      <c r="E1175"/>
+      <c r="D1175" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1175" t="n">
+        <v>0</v>
+      </c>
       <c r="F1175" t="n">
         <v>6.33</v>
       </c>
@@ -51886,8 +52484,12 @@
       <c r="C1184" t="n">
         <v>0.115</v>
       </c>
-      <c r="D1184"/>
-      <c r="E1184"/>
+      <c r="D1184" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1184" t="n">
+        <v>0</v>
+      </c>
       <c r="F1184" t="n">
         <v>7.18</v>
       </c>
@@ -51920,8 +52522,12 @@
       <c r="C1185" t="n">
         <v>0.049</v>
       </c>
-      <c r="D1185"/>
-      <c r="E1185"/>
+      <c r="D1185" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1185" t="n">
+        <v>0</v>
+      </c>
       <c r="F1185" t="n">
         <v>5.85</v>
       </c>
@@ -51954,8 +52560,12 @@
       <c r="C1186" t="n">
         <v>0.045</v>
       </c>
-      <c r="D1186"/>
-      <c r="E1186"/>
+      <c r="D1186" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1186" t="n">
+        <v>0</v>
+      </c>
       <c r="F1186" t="n">
         <v>6.4</v>
       </c>
@@ -51988,8 +52598,12 @@
       <c r="C1187" t="n">
         <v>0.049</v>
       </c>
-      <c r="D1187"/>
-      <c r="E1187"/>
+      <c r="D1187" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1187" t="n">
+        <v>0</v>
+      </c>
       <c r="F1187" t="n">
         <v>9.03</v>
       </c>
@@ -52668,8 +53282,12 @@
       <c r="C1205" t="n">
         <v>0.041</v>
       </c>
-      <c r="D1205"/>
-      <c r="E1205"/>
+      <c r="D1205" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1205" t="n">
+        <v>0</v>
+      </c>
       <c r="F1205" t="n">
         <v>17.24</v>
       </c>
@@ -52854,8 +53472,12 @@
       <c r="C1210" t="n">
         <v>0.032</v>
       </c>
-      <c r="D1210"/>
-      <c r="E1210"/>
+      <c r="D1210" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1210" t="n">
+        <v>0</v>
+      </c>
       <c r="F1210" t="n">
         <v>10.64</v>
       </c>
@@ -53572,8 +54194,12 @@
       <c r="C1229" t="n">
         <v>0.07</v>
       </c>
-      <c r="D1229"/>
-      <c r="E1229"/>
+      <c r="D1229" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1229" t="n">
+        <v>0</v>
+      </c>
       <c r="F1229" t="n">
         <v>8.44</v>
       </c>
@@ -54100,8 +54726,12 @@
       <c r="C1243" t="n">
         <v>0.034</v>
       </c>
-      <c r="D1243"/>
-      <c r="E1243"/>
+      <c r="D1243" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1243" t="n">
+        <v>0</v>
+      </c>
       <c r="F1243" t="n">
         <v>7.43</v>
       </c>
@@ -54210,8 +54840,12 @@
       <c r="C1246" t="n">
         <v>0.051</v>
       </c>
-      <c r="D1246"/>
-      <c r="E1246"/>
+      <c r="D1246" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1246" t="n">
+        <v>0</v>
+      </c>
       <c r="F1246" t="n">
         <v>7.56</v>
       </c>
@@ -54244,8 +54878,12 @@
       <c r="C1247" t="n">
         <v>0.032</v>
       </c>
-      <c r="D1247"/>
-      <c r="E1247"/>
+      <c r="D1247" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1247" t="n">
+        <v>0</v>
+      </c>
       <c r="F1247" t="n">
         <v>7.85</v>
       </c>
@@ -54972,8 +55610,12 @@
       <c r="C1267" t="n">
         <v>0.078</v>
       </c>
-      <c r="D1267"/>
-      <c r="E1267"/>
+      <c r="D1267" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1267" t="n">
+        <v>0</v>
+      </c>
       <c r="F1267" t="n">
         <v>7.69</v>
       </c>
@@ -55196,8 +55838,12 @@
       <c r="C1273" t="n">
         <v>0.083</v>
       </c>
-      <c r="D1273"/>
-      <c r="E1273"/>
+      <c r="D1273" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1273" t="n">
+        <v>0</v>
+      </c>
       <c r="F1273" t="n">
         <v>8.44</v>
       </c>
@@ -55382,8 +56028,12 @@
       <c r="C1278" t="n">
         <v>0.137</v>
       </c>
-      <c r="D1278"/>
-      <c r="E1278"/>
+      <c r="D1278" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1278" t="n">
+        <v>0</v>
+      </c>
       <c r="F1278" t="n">
         <v>12.46</v>
       </c>
@@ -55530,8 +56180,12 @@
       <c r="C1282" t="n">
         <v>0.038</v>
       </c>
-      <c r="D1282"/>
-      <c r="E1282"/>
+      <c r="D1282" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1282" t="n">
+        <v>0</v>
+      </c>
       <c r="F1282" t="n">
         <v>6.09</v>
       </c>
@@ -55564,8 +56218,12 @@
       <c r="C1283" t="n">
         <v>0.047</v>
       </c>
-      <c r="D1283"/>
-      <c r="E1283"/>
+      <c r="D1283" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1283" t="n">
+        <v>0</v>
+      </c>
       <c r="F1283" t="n">
         <v>7.02</v>
       </c>
@@ -56016,8 +56674,12 @@
       <c r="C1295" t="n">
         <v>0.033</v>
       </c>
-      <c r="D1295"/>
-      <c r="E1295"/>
+      <c r="D1295" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1295" t="n">
+        <v>0</v>
+      </c>
       <c r="F1295" t="n">
         <v>8.38</v>
       </c>
@@ -56050,8 +56712,12 @@
       <c r="C1296" t="n">
         <v>0.017</v>
       </c>
-      <c r="D1296"/>
-      <c r="E1296"/>
+      <c r="D1296" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1296" t="n">
+        <v>0</v>
+      </c>
       <c r="F1296" t="n">
         <v>8.68</v>
       </c>
@@ -56160,8 +56826,12 @@
       <c r="C1299" t="n">
         <v>0.031</v>
       </c>
-      <c r="D1299"/>
-      <c r="E1299"/>
+      <c r="D1299" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1299" t="n">
+        <v>0</v>
+      </c>
       <c r="F1299" t="n">
         <v>7.53</v>
       </c>
@@ -56384,8 +57054,12 @@
       <c r="C1305" t="n">
         <v>0.02</v>
       </c>
-      <c r="D1305"/>
-      <c r="E1305"/>
+      <c r="D1305" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1305" t="n">
+        <v>0</v>
+      </c>
       <c r="F1305" t="n">
         <v>11.56</v>
       </c>
@@ -56722,8 +57396,12 @@
       <c r="C1314" t="n">
         <v>0.059</v>
       </c>
-      <c r="D1314"/>
-      <c r="E1314"/>
+      <c r="D1314" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1314" t="n">
+        <v>0</v>
+      </c>
       <c r="F1314" t="n">
         <v>7.63</v>
       </c>
@@ -56870,8 +57548,12 @@
       <c r="C1318" t="n">
         <v>0.172</v>
       </c>
-      <c r="D1318"/>
-      <c r="E1318"/>
+      <c r="D1318" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1318" t="n">
+        <v>0</v>
+      </c>
       <c r="F1318" t="n">
         <v>4.11</v>
       </c>
@@ -56904,8 +57586,12 @@
       <c r="C1319" t="n">
         <v>0.11</v>
       </c>
-      <c r="D1319"/>
-      <c r="E1319"/>
+      <c r="D1319" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1319" t="n">
+        <v>0</v>
+      </c>
       <c r="F1319" t="n">
         <v>4.09</v>
       </c>
@@ -57090,8 +57776,12 @@
       <c r="C1324" t="n">
         <v>0.06</v>
       </c>
-      <c r="D1324"/>
-      <c r="E1324"/>
+      <c r="D1324" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1324" t="n">
+        <v>0</v>
+      </c>
       <c r="F1324" t="n">
         <v>7.38</v>
       </c>
@@ -57124,8 +57814,12 @@
       <c r="C1325" t="n">
         <v>0.086</v>
       </c>
-      <c r="D1325"/>
-      <c r="E1325"/>
+      <c r="D1325" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1325" t="n">
+        <v>0</v>
+      </c>
       <c r="F1325" t="n">
         <v>5.48</v>
       </c>
@@ -57196,8 +57890,12 @@
       <c r="C1327" t="n">
         <v>0.043</v>
       </c>
-      <c r="D1327"/>
-      <c r="E1327"/>
+      <c r="D1327" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1327" t="n">
+        <v>0</v>
+      </c>
       <c r="F1327" t="n">
         <v>6.8</v>
       </c>
@@ -57230,8 +57928,12 @@
       <c r="C1328" t="n">
         <v>0.058</v>
       </c>
-      <c r="D1328"/>
-      <c r="E1328"/>
+      <c r="D1328" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1328" t="n">
+        <v>0</v>
+      </c>
       <c r="F1328" t="n">
         <v>6.56</v>
       </c>
@@ -57264,8 +57966,12 @@
       <c r="C1329" t="n">
         <v>0.046</v>
       </c>
-      <c r="D1329"/>
-      <c r="E1329"/>
+      <c r="D1329" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1329" t="n">
+        <v>0</v>
+      </c>
       <c r="F1329" t="n">
         <v>9.78</v>
       </c>
@@ -57336,8 +58042,12 @@
       <c r="C1331" t="n">
         <v>0.054</v>
       </c>
-      <c r="D1331"/>
-      <c r="E1331"/>
+      <c r="D1331" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1331" t="n">
+        <v>0</v>
+      </c>
       <c r="F1331" t="n">
         <v>7.27</v>
       </c>
@@ -57370,8 +58080,12 @@
       <c r="C1332" t="n">
         <v>0.118</v>
       </c>
-      <c r="D1332"/>
-      <c r="E1332"/>
+      <c r="D1332" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1332" t="n">
+        <v>0</v>
+      </c>
       <c r="F1332" t="n">
         <v>7.44</v>
       </c>
@@ -57404,8 +58118,12 @@
       <c r="C1333" t="n">
         <v>0.118</v>
       </c>
-      <c r="D1333"/>
-      <c r="E1333"/>
+      <c r="D1333" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1333" t="n">
+        <v>0</v>
+      </c>
       <c r="F1333" t="n">
         <v>3.35</v>
       </c>
@@ -57438,8 +58156,12 @@
       <c r="C1334" t="n">
         <v>0.11</v>
       </c>
-      <c r="D1334"/>
-      <c r="E1334"/>
+      <c r="D1334" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1334" t="n">
+        <v>0</v>
+      </c>
       <c r="F1334" t="n">
         <v>1.6</v>
       </c>
@@ -58380,8 +59102,12 @@
       <c r="C1360" t="n">
         <v>0.081</v>
       </c>
-      <c r="D1360"/>
-      <c r="E1360"/>
+      <c r="D1360" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1360" t="n">
+        <v>0</v>
+      </c>
       <c r="F1360" t="n">
         <v>5.45</v>
       </c>
@@ -58704,8 +59430,12 @@
       <c r="C1369" t="n">
         <v>0.17</v>
       </c>
-      <c r="D1369"/>
-      <c r="E1369"/>
+      <c r="D1369" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1369" t="n">
+        <v>0</v>
+      </c>
       <c r="F1369" t="n">
         <v>7.61</v>
       </c>
@@ -59536,8 +60266,12 @@
       <c r="C1391" t="n">
         <v>0.148</v>
       </c>
-      <c r="D1391"/>
-      <c r="E1391"/>
+      <c r="D1391" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1391" t="n">
+        <v>0</v>
+      </c>
       <c r="F1391" t="n">
         <v>8.99</v>
       </c>
@@ -59646,8 +60380,12 @@
       <c r="C1394" t="n">
         <v>0.114</v>
       </c>
-      <c r="D1394"/>
-      <c r="E1394"/>
+      <c r="D1394" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1394" t="n">
+        <v>0</v>
+      </c>
       <c r="F1394" t="n">
         <v>7.55</v>
       </c>
@@ -59946,8 +60684,12 @@
       <c r="C1402" t="n">
         <v>0.13</v>
       </c>
-      <c r="D1402"/>
-      <c r="E1402"/>
+      <c r="D1402" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1402" t="n">
+        <v>0</v>
+      </c>
       <c r="F1402" t="n">
         <v>5.84</v>
       </c>
@@ -60018,8 +60760,12 @@
       <c r="C1404" t="n">
         <v>0.072</v>
       </c>
-      <c r="D1404"/>
-      <c r="E1404"/>
+      <c r="D1404" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1404" t="n">
+        <v>0</v>
+      </c>
       <c r="F1404" t="n">
         <v>7.42</v>
       </c>
@@ -60090,8 +60836,12 @@
       <c r="C1406" t="n">
         <v>0.11</v>
       </c>
-      <c r="D1406"/>
-      <c r="E1406"/>
+      <c r="D1406" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1406" t="n">
+        <v>0</v>
+      </c>
       <c r="F1406" t="n">
         <v>6.63</v>
       </c>
@@ -60390,8 +61140,12 @@
       <c r="C1414" t="n">
         <v>0.139</v>
       </c>
-      <c r="D1414"/>
-      <c r="E1414"/>
+      <c r="D1414" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1414" t="n">
+        <v>0</v>
+      </c>
       <c r="F1414" t="n">
         <v>6.78</v>
       </c>
@@ -60614,8 +61368,12 @@
       <c r="C1420" t="n">
         <v>0.114</v>
       </c>
-      <c r="D1420"/>
-      <c r="E1420"/>
+      <c r="D1420" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1420" t="n">
+        <v>0</v>
+      </c>
       <c r="F1420" t="n">
         <v>8.15</v>
       </c>
@@ -60686,8 +61444,12 @@
       <c r="C1422" t="n">
         <v>0.092</v>
       </c>
-      <c r="D1422"/>
-      <c r="E1422"/>
+      <c r="D1422" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1422" t="n">
+        <v>0</v>
+      </c>
       <c r="F1422" t="n">
         <v>5.99</v>
       </c>
@@ -60872,8 +61634,12 @@
       <c r="C1427" t="n">
         <v>0.113</v>
       </c>
-      <c r="D1427"/>
-      <c r="E1427"/>
+      <c r="D1427" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1427" t="n">
+        <v>0</v>
+      </c>
       <c r="F1427" t="n">
         <v>7.73</v>
       </c>
@@ -60944,8 +61710,12 @@
       <c r="C1429" t="n">
         <v>0.036</v>
       </c>
-      <c r="D1429"/>
-      <c r="E1429"/>
+      <c r="D1429" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1429" t="n">
+        <v>0</v>
+      </c>
       <c r="F1429" t="n">
         <v>8.72</v>
       </c>
@@ -61358,8 +62128,12 @@
       <c r="C1440" t="n">
         <v>0.037</v>
       </c>
-      <c r="D1440"/>
-      <c r="E1440"/>
+      <c r="D1440" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1440" t="n">
+        <v>0</v>
+      </c>
       <c r="F1440" t="n">
         <v>17.26</v>
       </c>
@@ -63216,8 +63990,12 @@
       <c r="C1489" t="n">
         <v>0.081</v>
       </c>
-      <c r="D1489"/>
-      <c r="E1489"/>
+      <c r="D1489" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1489" t="n">
+        <v>0</v>
+      </c>
       <c r="F1489" t="n">
         <v>10.09</v>
       </c>
@@ -63820,8 +64598,12 @@
       <c r="C1505" t="n">
         <v>0.076</v>
       </c>
-      <c r="D1505"/>
-      <c r="E1505"/>
+      <c r="D1505" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1505" t="n">
+        <v>0</v>
+      </c>
       <c r="F1505" t="n">
         <v>11.36</v>
       </c>
@@ -63892,8 +64674,12 @@
       <c r="C1507" t="n">
         <v>0.036</v>
       </c>
-      <c r="D1507"/>
-      <c r="E1507"/>
+      <c r="D1507" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1507" t="n">
+        <v>0</v>
+      </c>
       <c r="F1507" t="n">
         <v>12.89</v>
       </c>
@@ -64306,8 +65092,12 @@
       <c r="C1518" t="n">
         <v>0.027</v>
       </c>
-      <c r="D1518"/>
-      <c r="E1518"/>
+      <c r="D1518" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1518" t="n">
+        <v>0</v>
+      </c>
       <c r="F1518" t="n">
         <v>9.56</v>
       </c>
@@ -64907,7 +65697,9 @@
       <c r="B1534" t="n">
         <v>93.769</v>
       </c>
-      <c r="C1534"/>
+      <c r="C1534" t="n">
+        <v>0</v>
+      </c>
       <c r="D1534" t="n">
         <v>455</v>
       </c>
@@ -65005,7 +65797,9 @@
       <c r="B1537" t="n">
         <v>94.923</v>
       </c>
-      <c r="C1537"/>
+      <c r="C1537" t="n">
+        <v>0</v>
+      </c>
       <c r="D1537" t="n">
         <v>352.8</v>
       </c>
@@ -65383,7 +66177,9 @@
       <c r="B1547" t="n">
         <v>93.157</v>
       </c>
-      <c r="C1547"/>
+      <c r="C1547" t="n">
+        <v>0</v>
+      </c>
       <c r="D1547" t="n">
         <v>775.4</v>
       </c>
@@ -65457,7 +66253,9 @@
       <c r="B1549" t="n">
         <v>95.793</v>
       </c>
-      <c r="C1549"/>
+      <c r="C1549" t="n">
+        <v>0</v>
+      </c>
       <c r="D1549" t="n">
         <v>528.5</v>
       </c>
@@ -67655,7 +68453,9 @@
       <c r="B1608" t="n">
         <v>99.172</v>
       </c>
-      <c r="C1608"/>
+      <c r="C1608" t="n">
+        <v>0</v>
+      </c>
       <c r="D1608" t="n">
         <v>2060.2</v>
       </c>
@@ -67960,8 +68760,12 @@
       <c r="C1616" t="n">
         <v>0.014</v>
       </c>
-      <c r="D1616"/>
-      <c r="E1616"/>
+      <c r="D1616" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1616" t="n">
+        <v>0</v>
+      </c>
       <c r="F1616" t="n">
         <v>5.49</v>
       </c>
@@ -68143,7 +68947,9 @@
       <c r="B1621" t="n">
         <v>101.707</v>
       </c>
-      <c r="C1621"/>
+      <c r="C1621" t="n">
+        <v>0</v>
+      </c>
       <c r="D1621" t="n">
         <v>2878</v>
       </c>
@@ -69951,7 +70757,9 @@
       <c r="B1669" t="n">
         <v>94.93</v>
       </c>
-      <c r="C1669"/>
+      <c r="C1669" t="n">
+        <v>0</v>
+      </c>
       <c r="D1669" t="n">
         <v>66.2</v>
       </c>
@@ -69976,8 +70784,12 @@
       <c r="C1670" t="n">
         <v>0.01</v>
       </c>
-      <c r="D1670"/>
-      <c r="E1670"/>
+      <c r="D1670" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1670" t="n">
+        <v>0</v>
+      </c>
       <c r="F1670" t="n">
         <v>9.05</v>
       </c>
@@ -70086,8 +70898,12 @@
       <c r="C1673" t="n">
         <v>0.054</v>
       </c>
-      <c r="D1673"/>
-      <c r="E1673"/>
+      <c r="D1673" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1673" t="n">
+        <v>0</v>
+      </c>
       <c r="F1673" t="n">
         <v>9.13</v>
       </c>
@@ -70766,8 +71582,12 @@
       <c r="C1691" t="n">
         <v>0.139</v>
       </c>
-      <c r="D1691"/>
-      <c r="E1691"/>
+      <c r="D1691" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1691" t="n">
+        <v>0</v>
+      </c>
       <c r="F1691" t="n">
         <v>7.52</v>
       </c>
@@ -71318,8 +72138,12 @@
       <c r="C1706" t="n">
         <v>0.009</v>
       </c>
-      <c r="D1706"/>
-      <c r="E1706"/>
+      <c r="D1706" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1706" t="n">
+        <v>0</v>
+      </c>
       <c r="F1706" t="n">
         <v>8.57</v>
       </c>
@@ -71653,7 +72477,9 @@
       <c r="B1715" t="n">
         <v>93.558</v>
       </c>
-      <c r="C1715"/>
+      <c r="C1715" t="n">
+        <v>0</v>
+      </c>
       <c r="D1715" t="n">
         <v>24.2</v>
       </c>
@@ -71996,8 +72822,12 @@
       <c r="C1724" t="n">
         <v>0.017</v>
       </c>
-      <c r="D1724"/>
-      <c r="E1724"/>
+      <c r="D1724" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1724" t="n">
+        <v>0</v>
+      </c>
       <c r="F1724" t="n">
         <v>8.27</v>
       </c>
@@ -72828,8 +73658,12 @@
       <c r="C1746" t="n">
         <v>0.05</v>
       </c>
-      <c r="D1746"/>
-      <c r="E1746"/>
+      <c r="D1746" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1746" t="n">
+        <v>0</v>
+      </c>
       <c r="F1746" t="n">
         <v>7.2</v>
       </c>
@@ -73090,8 +73924,12 @@
       <c r="C1753" t="n">
         <v>0.115</v>
       </c>
-      <c r="D1753"/>
-      <c r="E1753"/>
+      <c r="D1753" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1753" t="n">
+        <v>0</v>
+      </c>
       <c r="F1753" t="n">
         <v>7.64</v>
       </c>
@@ -75524,8 +76362,12 @@
       <c r="C1819" t="n">
         <v>0.009</v>
       </c>
-      <c r="D1819"/>
-      <c r="E1819"/>
+      <c r="D1819" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1819" t="n">
+        <v>0</v>
+      </c>
       <c r="F1819"/>
       <c r="G1819"/>
       <c r="H1819"/>
@@ -75962,8 +76804,12 @@
       <c r="C1831" t="n">
         <v>0.003</v>
       </c>
-      <c r="D1831"/>
-      <c r="E1831"/>
+      <c r="D1831" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1831" t="n">
+        <v>0</v>
+      </c>
       <c r="F1831" t="n">
         <v>7.58</v>
       </c>
@@ -77309,7 +78155,9 @@
       <c r="B1867" t="n">
         <v>95.006</v>
       </c>
-      <c r="C1867"/>
+      <c r="C1867" t="n">
+        <v>0</v>
+      </c>
       <c r="D1867" t="n">
         <v>510.6</v>
       </c>
@@ -79987,7 +80835,9 @@
       <c r="B1939" t="n">
         <v>99.351</v>
       </c>
-      <c r="C1939"/>
+      <c r="C1939" t="n">
+        <v>0</v>
+      </c>
       <c r="D1939" t="n">
         <v>2997.2</v>
       </c>
@@ -80109,7 +80959,9 @@
       <c r="B1943" t="n">
         <v>99.458</v>
       </c>
-      <c r="C1943"/>
+      <c r="C1943" t="n">
+        <v>0</v>
+      </c>
       <c r="D1943" t="n">
         <v>2381.2</v>
       </c>
@@ -80718,8 +81570,12 @@
       <c r="C1959" t="n">
         <v>0.012</v>
       </c>
-      <c r="D1959"/>
-      <c r="E1959"/>
+      <c r="D1959" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1959" t="n">
+        <v>0</v>
+      </c>
       <c r="F1959" t="n">
         <v>4.85</v>
       </c>
@@ -83205,7 +84061,9 @@
       <c r="B2025" t="n">
         <v>92.248</v>
       </c>
-      <c r="C2025"/>
+      <c r="C2025" t="n">
+        <v>0</v>
+      </c>
       <c r="D2025" t="n">
         <v>856.4</v>
       </c>
@@ -83700,8 +84558,12 @@
       <c r="C2038" t="n">
         <v>0.008</v>
       </c>
-      <c r="D2038"/>
-      <c r="E2038"/>
+      <c r="D2038" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2038" t="n">
+        <v>0</v>
+      </c>
       <c r="F2038" t="n">
         <v>8.32</v>
       </c>
@@ -83772,8 +84634,12 @@
       <c r="C2040" t="n">
         <v>0.027</v>
       </c>
-      <c r="D2040"/>
-      <c r="E2040"/>
+      <c r="D2040" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2040" t="n">
+        <v>0</v>
+      </c>
       <c r="F2040" t="n">
         <v>9.18</v>
       </c>
@@ -83806,8 +84672,12 @@
       <c r="C2041" t="n">
         <v>0.008</v>
       </c>
-      <c r="D2041"/>
-      <c r="E2041"/>
+      <c r="D2041" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2041" t="n">
+        <v>0</v>
+      </c>
       <c r="F2041" t="n">
         <v>5.72</v>
       </c>
@@ -84524,8 +85394,12 @@
       <c r="C2060" t="n">
         <v>0.067</v>
       </c>
-      <c r="D2060"/>
-      <c r="E2060"/>
+      <c r="D2060" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2060" t="n">
+        <v>0</v>
+      </c>
       <c r="F2060" t="n">
         <v>19.65</v>
       </c>
@@ -84672,8 +85546,12 @@
       <c r="C2064" t="n">
         <v>0.074</v>
       </c>
-      <c r="D2064"/>
-      <c r="E2064"/>
+      <c r="D2064" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2064" t="n">
+        <v>0</v>
+      </c>
       <c r="F2064" t="n">
         <v>9.45</v>
       </c>
@@ -85048,8 +85926,12 @@
       <c r="C2074" t="n">
         <v>0.036</v>
       </c>
-      <c r="D2074"/>
-      <c r="E2074"/>
+      <c r="D2074" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2074" t="n">
+        <v>0</v>
+      </c>
       <c r="F2074" t="n">
         <v>8.21</v>
       </c>
@@ -85842,8 +86724,12 @@
       <c r="C2095" t="n">
         <v>0.093</v>
       </c>
-      <c r="D2095"/>
-      <c r="E2095"/>
+      <c r="D2095" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2095" t="n">
+        <v>0</v>
+      </c>
       <c r="F2095" t="n">
         <v>6.36</v>
       </c>
@@ -86522,8 +87408,12 @@
       <c r="C2113" t="n">
         <v>0.084</v>
       </c>
-      <c r="D2113"/>
-      <c r="E2113"/>
+      <c r="D2113" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2113" t="n">
+        <v>0</v>
+      </c>
       <c r="F2113" t="n">
         <v>7.52</v>
       </c>
@@ -87264,8 +88154,12 @@
       <c r="C2133" t="n">
         <v>0.064</v>
       </c>
-      <c r="D2133"/>
-      <c r="E2133"/>
+      <c r="D2133" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2133" t="n">
+        <v>0</v>
+      </c>
       <c r="F2133" t="n">
         <v>8.77</v>
       </c>
@@ -87854,8 +88748,12 @@
       <c r="C2149" t="n">
         <v>0.018</v>
       </c>
-      <c r="D2149"/>
-      <c r="E2149"/>
+      <c r="D2149" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2149" t="n">
+        <v>0</v>
+      </c>
       <c r="F2149" t="n">
         <v>12.19</v>
       </c>
@@ -90724,8 +91622,12 @@
       <c r="C2225" t="n">
         <v>0.031</v>
       </c>
-      <c r="D2225"/>
-      <c r="E2225"/>
+      <c r="D2225" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2225" t="n">
+        <v>0</v>
+      </c>
       <c r="F2225" t="n">
         <v>5.89</v>
       </c>
@@ -91252,8 +92154,12 @@
       <c r="C2239" t="n">
         <v>0.048</v>
       </c>
-      <c r="D2239"/>
-      <c r="E2239"/>
+      <c r="D2239" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2239" t="n">
+        <v>0</v>
+      </c>
       <c r="F2239" t="n">
         <v>10.09</v>
       </c>
@@ -91476,8 +92382,12 @@
       <c r="C2245" t="n">
         <v>0.022</v>
       </c>
-      <c r="D2245"/>
-      <c r="E2245"/>
+      <c r="D2245" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2245" t="n">
+        <v>0</v>
+      </c>
       <c r="F2245" t="n">
         <v>6.25</v>
       </c>
@@ -92153,7 +93063,9 @@
       <c r="B2263" t="n">
         <v>94.778</v>
       </c>
-      <c r="C2263"/>
+      <c r="C2263" t="n">
+        <v>0</v>
+      </c>
       <c r="D2263" t="n">
         <v>681.8</v>
       </c>
@@ -92192,8 +93104,12 @@
       <c r="C2264" t="n">
         <v>0.006</v>
       </c>
-      <c r="D2264"/>
-      <c r="E2264"/>
+      <c r="D2264" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2264" t="n">
+        <v>0</v>
+      </c>
       <c r="F2264" t="n">
         <v>7.46</v>
       </c>
@@ -92668,8 +93584,12 @@
       <c r="C2277" t="n">
         <v>0.036</v>
       </c>
-      <c r="D2277"/>
-      <c r="E2277"/>
+      <c r="D2277" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2277" t="n">
+        <v>0</v>
+      </c>
       <c r="F2277" t="n">
         <v>6.58</v>
       </c>
@@ -92816,8 +93736,12 @@
       <c r="C2281" t="n">
         <v>0.038</v>
       </c>
-      <c r="D2281"/>
-      <c r="E2281"/>
+      <c r="D2281" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2281" t="n">
+        <v>0</v>
+      </c>
       <c r="F2281" t="n">
         <v>7.1</v>
       </c>
@@ -93976,8 +94900,12 @@
       <c r="C2312" t="n">
         <v>0.008</v>
       </c>
-      <c r="D2312"/>
-      <c r="E2312"/>
+      <c r="D2312" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2312" t="n">
+        <v>0</v>
+      </c>
       <c r="F2312" t="n">
         <v>6.5</v>
       </c>
@@ -94352,8 +95280,12 @@
       <c r="C2322" t="n">
         <v>0.048</v>
       </c>
-      <c r="D2322"/>
-      <c r="E2322"/>
+      <c r="D2322" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2322" t="n">
+        <v>0</v>
+      </c>
       <c r="F2322" t="n">
         <v>5.99</v>
       </c>
@@ -94538,8 +95470,12 @@
       <c r="C2327" t="n">
         <v>0.047</v>
       </c>
-      <c r="D2327"/>
-      <c r="E2327"/>
+      <c r="D2327" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2327" t="n">
+        <v>0</v>
+      </c>
       <c r="F2327" t="n">
         <v>6.27</v>
       </c>
@@ -94762,8 +95698,12 @@
       <c r="C2333" t="n">
         <v>0.036</v>
       </c>
-      <c r="D2333"/>
-      <c r="E2333"/>
+      <c r="D2333" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2333" t="n">
+        <v>0</v>
+      </c>
       <c r="F2333" t="n">
         <v>6.7</v>
       </c>
@@ -94910,8 +95850,12 @@
       <c r="C2337" t="n">
         <v>0.042</v>
       </c>
-      <c r="D2337"/>
-      <c r="E2337"/>
+      <c r="D2337" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2337" t="n">
+        <v>0</v>
+      </c>
       <c r="F2337" t="n">
         <v>7.37</v>
       </c>
@@ -95970,8 +96914,12 @@
       <c r="C2365" t="n">
         <v>0.023</v>
       </c>
-      <c r="D2365"/>
-      <c r="E2365"/>
+      <c r="D2365" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2365" t="n">
+        <v>0</v>
+      </c>
       <c r="F2365" t="n">
         <v>7.65</v>
       </c>
@@ -96004,8 +96952,12 @@
       <c r="C2366" t="n">
         <v>0.144</v>
       </c>
-      <c r="D2366"/>
-      <c r="E2366"/>
+      <c r="D2366" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2366" t="n">
+        <v>0</v>
+      </c>
       <c r="F2366" t="n">
         <v>7.34</v>
       </c>
@@ -96646,8 +97598,12 @@
       <c r="C2383" t="n">
         <v>0.04</v>
       </c>
-      <c r="D2383"/>
-      <c r="E2383"/>
+      <c r="D2383" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2383" t="n">
+        <v>0</v>
+      </c>
       <c r="F2383" t="n">
         <v>14.78</v>
       </c>
@@ -96794,8 +97750,12 @@
       <c r="C2387" t="n">
         <v>0.057</v>
       </c>
-      <c r="D2387"/>
-      <c r="E2387"/>
+      <c r="D2387" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2387" t="n">
+        <v>0</v>
+      </c>
       <c r="F2387" t="n">
         <v>9.2</v>
       </c>
@@ -97588,8 +98548,12 @@
       <c r="C2408" t="n">
         <v>0.09</v>
       </c>
-      <c r="D2408"/>
-      <c r="E2408"/>
+      <c r="D2408" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2408" t="n">
+        <v>0</v>
+      </c>
       <c r="F2408" t="n">
         <v>12.68</v>
       </c>
@@ -97660,8 +98624,12 @@
       <c r="C2410" t="n">
         <v>0.049</v>
       </c>
-      <c r="D2410"/>
-      <c r="E2410"/>
+      <c r="D2410" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2410" t="n">
+        <v>0</v>
+      </c>
       <c r="F2410" t="n">
         <v>15.42</v>
       </c>
@@ -98150,8 +99118,12 @@
       <c r="C2423" t="n">
         <v>0.036</v>
       </c>
-      <c r="D2423"/>
-      <c r="E2423"/>
+      <c r="D2423" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2423" t="n">
+        <v>0</v>
+      </c>
       <c r="F2423" t="n">
         <v>10.61</v>
       </c>
@@ -99210,8 +100182,12 @@
       <c r="C2451" t="n">
         <v>0.058</v>
       </c>
-      <c r="D2451"/>
-      <c r="E2451"/>
+      <c r="D2451" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2451" t="n">
+        <v>0</v>
+      </c>
       <c r="F2451" t="n">
         <v>8.36</v>
       </c>
@@ -99596,8 +100572,12 @@
       <c r="C2462" t="n">
         <v>0.07</v>
       </c>
-      <c r="D2462"/>
-      <c r="E2462"/>
+      <c r="D2462" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2462" t="n">
+        <v>0</v>
+      </c>
       <c r="F2462" t="n">
         <v>6.86</v>
       </c>
@@ -100832,8 +101812,12 @@
       <c r="C2495" t="n">
         <v>0.027</v>
       </c>
-      <c r="D2495"/>
-      <c r="E2495"/>
+      <c r="D2495" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2495" t="n">
+        <v>0</v>
+      </c>
       <c r="F2495" t="n">
         <v>5.9</v>
       </c>
@@ -100904,8 +101888,12 @@
       <c r="C2497" t="n">
         <v>0.02</v>
       </c>
-      <c r="D2497"/>
-      <c r="E2497"/>
+      <c r="D2497" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2497" t="n">
+        <v>0</v>
+      </c>
       <c r="F2497" t="n">
         <v>6.95</v>
       </c>
@@ -101280,8 +102268,12 @@
       <c r="C2507" t="n">
         <v>0.017</v>
       </c>
-      <c r="D2507"/>
-      <c r="E2507"/>
+      <c r="D2507" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2507" t="n">
+        <v>0</v>
+      </c>
       <c r="F2507" t="n">
         <v>8.12</v>
       </c>
@@ -101352,8 +102344,12 @@
       <c r="C2509" t="n">
         <v>0.047</v>
       </c>
-      <c r="D2509"/>
-      <c r="E2509"/>
+      <c r="D2509" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2509" t="n">
+        <v>0</v>
+      </c>
       <c r="F2509" t="n">
         <v>7.59</v>
       </c>
@@ -101424,8 +102420,12 @@
       <c r="C2511" t="n">
         <v>0.075</v>
       </c>
-      <c r="D2511"/>
-      <c r="E2511"/>
+      <c r="D2511" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2511" t="n">
+        <v>0</v>
+      </c>
       <c r="F2511" t="n">
         <v>5.45</v>
       </c>
@@ -101458,8 +102458,12 @@
       <c r="C2512" t="n">
         <v>0.069</v>
       </c>
-      <c r="D2512"/>
-      <c r="E2512"/>
+      <c r="D2512" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2512" t="n">
+        <v>0</v>
+      </c>
       <c r="F2512" t="n">
         <v>6.13</v>
       </c>
@@ -101606,8 +102610,12 @@
       <c r="C2516" t="n">
         <v>0.021</v>
       </c>
-      <c r="D2516"/>
-      <c r="E2516"/>
+      <c r="D2516" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2516" t="n">
+        <v>0</v>
+      </c>
       <c r="F2516" t="n">
         <v>8.67</v>
       </c>
@@ -101716,8 +102724,12 @@
       <c r="C2519" t="n">
         <v>0.03</v>
       </c>
-      <c r="D2519"/>
-      <c r="E2519"/>
+      <c r="D2519" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2519" t="n">
+        <v>0</v>
+      </c>
       <c r="F2519" t="n">
         <v>9.55</v>
       </c>
@@ -101750,8 +102762,12 @@
       <c r="C2520" t="n">
         <v>0.059</v>
       </c>
-      <c r="D2520"/>
-      <c r="E2520"/>
+      <c r="D2520" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2520" t="n">
+        <v>0</v>
+      </c>
       <c r="F2520" t="n">
         <v>5.15</v>
       </c>
@@ -101936,8 +102952,12 @@
       <c r="C2525" t="n">
         <v>0.021</v>
       </c>
-      <c r="D2525"/>
-      <c r="E2525"/>
+      <c r="D2525" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2525" t="n">
+        <v>0</v>
+      </c>
       <c r="F2525" t="n">
         <v>6.86</v>
       </c>
@@ -102008,8 +103028,12 @@
       <c r="C2527" t="n">
         <v>0.049</v>
       </c>
-      <c r="D2527"/>
-      <c r="E2527"/>
+      <c r="D2527" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2527" t="n">
+        <v>0</v>
+      </c>
       <c r="F2527" t="n">
         <v>6.31</v>
       </c>
@@ -102042,8 +103066,12 @@
       <c r="C2528" t="n">
         <v>0.047</v>
       </c>
-      <c r="D2528"/>
-      <c r="E2528"/>
+      <c r="D2528" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2528" t="n">
+        <v>0</v>
+      </c>
       <c r="F2528" t="n">
         <v>5.61</v>
       </c>
@@ -102076,8 +103104,12 @@
       <c r="C2529" t="n">
         <v>0.057</v>
       </c>
-      <c r="D2529"/>
-      <c r="E2529"/>
+      <c r="D2529" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2529" t="n">
+        <v>0</v>
+      </c>
       <c r="F2529" t="n">
         <v>6.54</v>
       </c>
@@ -102110,8 +103142,12 @@
       <c r="C2530" t="n">
         <v>0</v>
       </c>
-      <c r="D2530"/>
-      <c r="E2530"/>
+      <c r="D2530" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2530" t="n">
+        <v>0</v>
+      </c>
       <c r="F2530" t="n">
         <v>5.86</v>
       </c>
@@ -102220,8 +103256,12 @@
       <c r="C2533" t="n">
         <v>0.024</v>
       </c>
-      <c r="D2533"/>
-      <c r="E2533"/>
+      <c r="D2533" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2533" t="n">
+        <v>0</v>
+      </c>
       <c r="F2533" t="n">
         <v>6.92</v>
       </c>
@@ -102292,8 +103332,12 @@
       <c r="C2535" t="n">
         <v>0.027</v>
       </c>
-      <c r="D2535"/>
-      <c r="E2535"/>
+      <c r="D2535" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2535" t="n">
+        <v>0</v>
+      </c>
       <c r="F2535" t="n">
         <v>7.19</v>
       </c>
@@ -102630,8 +103674,12 @@
       <c r="C2544" t="n">
         <v>0.056</v>
       </c>
-      <c r="D2544"/>
-      <c r="E2544"/>
+      <c r="D2544" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2544" t="n">
+        <v>0</v>
+      </c>
       <c r="F2544" t="n">
         <v>7.26</v>
       </c>
@@ -102664,8 +103712,12 @@
       <c r="C2545" t="n">
         <v>0.038</v>
       </c>
-      <c r="D2545"/>
-      <c r="E2545"/>
+      <c r="D2545" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2545" t="n">
+        <v>0</v>
+      </c>
       <c r="F2545" t="n">
         <v>7.74</v>
       </c>
@@ -102698,8 +103750,12 @@
       <c r="C2546" t="n">
         <v>0.018</v>
       </c>
-      <c r="D2546"/>
-      <c r="E2546"/>
+      <c r="D2546" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2546" t="n">
+        <v>0</v>
+      </c>
       <c r="F2546" t="n">
         <v>8.26</v>
       </c>
@@ -102960,8 +104016,12 @@
       <c r="C2553" t="n">
         <v>0.049</v>
       </c>
-      <c r="D2553"/>
-      <c r="E2553"/>
+      <c r="D2553" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2553" t="n">
+        <v>0</v>
+      </c>
       <c r="F2553" t="n">
         <v>6.41</v>
       </c>
@@ -103146,8 +104206,12 @@
       <c r="C2558" t="n">
         <v>0.046</v>
       </c>
-      <c r="D2558"/>
-      <c r="E2558"/>
+      <c r="D2558" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2558" t="n">
+        <v>0</v>
+      </c>
       <c r="F2558" t="n">
         <v>8.57</v>
       </c>
@@ -103218,8 +104282,12 @@
       <c r="C2560" t="n">
         <v>0.007</v>
       </c>
-      <c r="D2560"/>
-      <c r="E2560"/>
+      <c r="D2560" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2560" t="n">
+        <v>0</v>
+      </c>
       <c r="F2560" t="n">
         <v>8.16</v>
       </c>
@@ -103252,8 +104320,12 @@
       <c r="C2561" t="n">
         <v>0.025</v>
       </c>
-      <c r="D2561"/>
-      <c r="E2561"/>
+      <c r="D2561" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2561" t="n">
+        <v>0</v>
+      </c>
       <c r="F2561" t="n">
         <v>4.56</v>
       </c>

</xml_diff>